<commit_message>
feat: varredura e fechamento de 12 a 18 e inicio de 19 a 20 com 67 lojas e 5276 pedidos resgatados
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-01).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-01).xlsx
@@ -938,13 +938,13 @@
     <t>215</t>
   </si>
   <si>
-    <t>26</t>
+    <t>24</t>
   </si>
   <si>
-    <t>R$ 4.622,53</t>
+    <t>R$ 4.631,12</t>
   </si>
   <si>
-    <t>50.6</t>
+    <t>50.7</t>
   </si>
   <si>
     <t>31.9</t>
@@ -953,16 +953,16 @@
     <t>5.06</t>
   </si>
   <si>
-    <t>19.4</t>
+    <t>19.5</t>
   </si>
   <si>
-    <t>7.6</t>
+    <t>7.7</t>
   </si>
   <si>
     <t>6.4</t>
   </si>
   <si>
-    <t>41.3%</t>
+    <t>41.6%</t>
   </si>
   <si>
     <t>18.0%</t>
@@ -10288,7 +10288,7 @@
         <v>19618</v>
       </c>
       <c r="B58" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C58" s="4">
         <v>51</v>
@@ -10318,18 +10318,30 @@
         <v>58</v>
       </c>
       <c r="L58" s="4"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="6"/>
+      <c r="M58" s="5">
+        <v>5794.1700000000001</v>
+      </c>
+      <c r="N58" s="6">
+        <v>71</v>
+      </c>
       <c r="O58" s="6">
         <v>52</v>
       </c>
-      <c r="P58" s="7"/>
-      <c r="Q58" s="8"/>
-      <c r="R58" s="8"/>
+      <c r="P58" s="7">
+        <v>4.0748723076923072</v>
+      </c>
+      <c r="Q58" s="8">
+        <v>24.092628846153847</v>
+      </c>
+      <c r="R58" s="8">
+        <v>13.158332692307692</v>
+      </c>
       <c r="S58" s="8">
         <v>7</v>
       </c>
-      <c r="T58" s="9"/>
+      <c r="T58" s="9">
+        <v>0.23076923076923078</v>
+      </c>
       <c r="U58" s="9">
         <v>0.096153846153846159</v>
       </c>
@@ -14941,7 +14953,7 @@
         <v>19693</v>
       </c>
       <c r="B89" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C89" s="4">
         <v>51</v>
@@ -14969,14 +14981,26 @@
         <v>58</v>
       </c>
       <c r="L89" s="4"/>
-      <c r="M89" s="5"/>
-      <c r="N89" s="6"/>
+      <c r="M89" s="5">
+        <v>5082.4700000000003</v>
+      </c>
+      <c r="N89" s="6">
+        <v>46</v>
+      </c>
       <c r="O89" s="6"/>
-      <c r="P89" s="7"/>
-      <c r="Q89" s="8"/>
-      <c r="R89" s="8"/>
+      <c r="P89" s="7">
+        <v>5.2607645833333327</v>
+      </c>
+      <c r="Q89" s="8">
+        <v>29.250596428571431</v>
+      </c>
+      <c r="R89" s="8">
+        <v>15.513689285714287</v>
+      </c>
       <c r="S89" s="8"/>
-      <c r="T89" s="9"/>
+      <c r="T89" s="9">
+        <v>0.10714285714285714</v>
+      </c>
       <c r="U89" s="9"/>
       <c r="V89" s="9"/>
       <c r="W89" s="9"/>
@@ -29425,7 +29449,7 @@
         <v>19923</v>
       </c>
       <c r="B185" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c t="s" r="C185" s="4">
         <v>51</v>
@@ -32133,7 +32157,7 @@
         <v>19957</v>
       </c>
       <c r="B203" s="3">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c t="s" r="C203" s="4">
         <v>51</v>
@@ -33766,7 +33790,7 @@
         <v>19980</v>
       </c>
       <c r="B216" s="3">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c t="s" r="C216" s="4">
         <v>51</v>

</xml_diff>

<commit_message>
feat: varredura e atualizacao com dias 21 e 22/10 avancando semana para 19 a 22 com 165 recuperacoes e 8978 pedidos resgatados
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-01).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-01).xlsx
@@ -938,37 +938,37 @@
     <t>215</t>
   </si>
   <si>
-    <t>24</t>
+    <t>21</t>
   </si>
   <si>
-    <t>R$ 4.631,12</t>
+    <t>R$ 4.598,43</t>
   </si>
   <si>
-    <t>50.7</t>
+    <t>50.4</t>
   </si>
   <si>
-    <t>31.9</t>
+    <t>31.8</t>
   </si>
   <si>
-    <t>5.06</t>
+    <t>5.04</t>
   </si>
   <si>
-    <t>19.5</t>
+    <t>19.4</t>
   </si>
   <si>
-    <t>7.7</t>
+    <t>7.6</t>
   </si>
   <si>
-    <t>6.4</t>
+    <t>6.5</t>
   </si>
   <si>
-    <t>41.6%</t>
+    <t>41.9%</t>
   </si>
   <si>
-    <t>18.0%</t>
+    <t>18.1%</t>
   </si>
   <si>
-    <t>1.9%</t>
+    <t>1.8%</t>
   </si>
   <si>
     <t>0.2%</t>
@@ -989,13 +989,13 @@
     <t>2.8%</t>
   </si>
   <si>
-    <t>3.9%</t>
+    <t>4.0%</t>
   </si>
   <si>
-    <t>1351.0</t>
+    <t>1372.0</t>
   </si>
   <si>
-    <t>1103.0</t>
+    <t>1122.0</t>
   </si>
   <si>
     <t>114.0</t>
@@ -1004,7 +1004,7 @@
     <t>14.0</t>
   </si>
   <si>
-    <t>299.0</t>
+    <t>305.0</t>
   </si>
   <si>
     <t>69.0</t>
@@ -1013,13 +1013,13 @@
     <t>9.0</t>
   </si>
   <si>
-    <t>398.0</t>
+    <t>403.0</t>
   </si>
   <si>
     <t>172.0</t>
   </si>
   <si>
-    <t>238.0</t>
+    <t>248.0</t>
   </si>
   <si>
     <t>0.8%</t>
@@ -24301,7 +24301,7 @@
         <v>19821</v>
       </c>
       <c r="B151" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C151" s="4">
         <v>51</v>
@@ -24331,35 +24331,93 @@
         <v>58</v>
       </c>
       <c r="L151" s="4"/>
-      <c r="M151" s="5"/>
-      <c r="N151" s="6"/>
-      <c r="O151" s="6"/>
-      <c r="P151" s="7"/>
-      <c r="Q151" s="8"/>
-      <c r="R151" s="8"/>
-      <c r="S151" s="8"/>
-      <c r="T151" s="9"/>
-      <c r="U151" s="9"/>
-      <c r="V151" s="9"/>
-      <c r="W151" s="9"/>
-      <c r="X151" s="9"/>
-      <c r="Y151" s="9"/>
-      <c r="Z151" s="9"/>
-      <c r="AA151" s="9"/>
-      <c r="AB151" s="9"/>
-      <c r="AC151" s="9"/>
-      <c r="AD151" s="6"/>
-      <c r="AE151" s="6"/>
-      <c r="AF151" s="6"/>
-      <c r="AG151" s="6"/>
-      <c r="AH151" s="6"/>
-      <c r="AI151" s="6"/>
-      <c r="AJ151" s="6"/>
-      <c r="AK151" s="6"/>
-      <c r="AL151" s="6"/>
-      <c r="AM151" s="6"/>
-      <c r="AN151" s="9"/>
-      <c r="AO151" s="6"/>
+      <c r="M151" s="5">
+        <v>3124.9000000000001</v>
+      </c>
+      <c r="N151" s="6">
+        <v>43</v>
+      </c>
+      <c r="O151" s="6">
+        <v>40</v>
+      </c>
+      <c r="P151" s="7">
+        <v>3.0522727272727277</v>
+      </c>
+      <c r="Q151" s="8">
+        <v>12.690417499999999</v>
+      </c>
+      <c r="R151" s="8">
+        <v>2.8070824999999999</v>
+      </c>
+      <c r="S151" s="8">
+        <v>7</v>
+      </c>
+      <c r="T151" s="9">
+        <v>0.90000000000000002</v>
+      </c>
+      <c r="U151" s="9">
+        <v>0.25</v>
+      </c>
+      <c r="V151" s="9">
+        <v>0</v>
+      </c>
+      <c r="W151" s="9">
+        <v>0</v>
+      </c>
+      <c r="X151" s="9">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="Y151" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z151" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA151" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB151" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC151" s="9">
+        <v>0.14999999999999999</v>
+      </c>
+      <c r="AD151" s="6">
+        <v>12</v>
+      </c>
+      <c r="AE151" s="6">
+        <v>10</v>
+      </c>
+      <c r="AF151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH151" s="6">
+        <v>6</v>
+      </c>
+      <c r="AI151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL151" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM151" s="6">
+        <v>6</v>
+      </c>
+      <c r="AN151" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO151" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP151" s="4">
         <v>58</v>
       </c>
@@ -25183,7 +25241,7 @@
         <v>19855</v>
       </c>
       <c r="B157" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C157" s="4">
         <v>51</v>
@@ -25213,35 +25271,93 @@
         <v>58</v>
       </c>
       <c r="L157" s="4"/>
-      <c r="M157" s="5"/>
-      <c r="N157" s="6"/>
-      <c r="O157" s="6"/>
-      <c r="P157" s="7"/>
-      <c r="Q157" s="8"/>
-      <c r="R157" s="8"/>
-      <c r="S157" s="8"/>
-      <c r="T157" s="9"/>
-      <c r="U157" s="9"/>
-      <c r="V157" s="9"/>
-      <c r="W157" s="9"/>
-      <c r="X157" s="9"/>
-      <c r="Y157" s="9"/>
-      <c r="Z157" s="9"/>
-      <c r="AA157" s="9"/>
-      <c r="AB157" s="9"/>
-      <c r="AC157" s="9"/>
-      <c r="AD157" s="6"/>
-      <c r="AE157" s="6"/>
-      <c r="AF157" s="6"/>
-      <c r="AG157" s="6"/>
-      <c r="AH157" s="6"/>
-      <c r="AI157" s="6"/>
-      <c r="AJ157" s="6"/>
-      <c r="AK157" s="6"/>
-      <c r="AL157" s="6"/>
-      <c r="AM157" s="6"/>
-      <c r="AN157" s="9"/>
-      <c r="AO157" s="6"/>
+      <c r="M157" s="5">
+        <v>2308.9099999999999</v>
+      </c>
+      <c r="N157" s="6">
+        <v>28</v>
+      </c>
+      <c r="O157" s="6">
+        <v>22</v>
+      </c>
+      <c r="P157" s="7">
+        <v>6.3214285714285712</v>
+      </c>
+      <c r="Q157" s="8">
+        <v>15.785604545454545</v>
+      </c>
+      <c r="R157" s="8">
+        <v>3.9657388888888891</v>
+      </c>
+      <c r="S157" s="8">
+        <v>7</v>
+      </c>
+      <c r="T157" s="9">
+        <v>0.31818181818181818</v>
+      </c>
+      <c r="U157" s="9">
+        <v>0.40909090909090912</v>
+      </c>
+      <c r="V157" s="9">
+        <v>0</v>
+      </c>
+      <c r="W157" s="9">
+        <v>0</v>
+      </c>
+      <c r="X157" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y157" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z157" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA157" s="9">
+        <v>0.22727272727272727</v>
+      </c>
+      <c r="AB157" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC157" s="9">
+        <v>0.18181818181818182</v>
+      </c>
+      <c r="AD157" s="6">
+        <v>9</v>
+      </c>
+      <c r="AE157" s="6">
+        <v>9</v>
+      </c>
+      <c r="AF157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK157" s="6">
+        <v>5</v>
+      </c>
+      <c r="AL157" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM157" s="6">
+        <v>4</v>
+      </c>
+      <c r="AN157" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO157" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP157" s="4">
         <v>58</v>
       </c>
@@ -26375,7 +26491,7 @@
         <v>19877</v>
       </c>
       <c r="B165" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C165" s="4">
         <v>51</v>
@@ -26405,35 +26521,93 @@
         <v>58</v>
       </c>
       <c r="L165" s="4"/>
-      <c r="M165" s="5"/>
-      <c r="N165" s="6"/>
-      <c r="O165" s="6"/>
-      <c r="P165" s="7"/>
-      <c r="Q165" s="8"/>
-      <c r="R165" s="8"/>
-      <c r="S165" s="8"/>
-      <c r="T165" s="9"/>
-      <c r="U165" s="9"/>
-      <c r="V165" s="9"/>
-      <c r="W165" s="9"/>
-      <c r="X165" s="9"/>
-      <c r="Y165" s="9"/>
-      <c r="Z165" s="9"/>
-      <c r="AA165" s="9"/>
-      <c r="AB165" s="9"/>
-      <c r="AC165" s="9"/>
-      <c r="AD165" s="6"/>
-      <c r="AE165" s="6"/>
-      <c r="AF165" s="6"/>
-      <c r="AG165" s="6"/>
-      <c r="AH165" s="6"/>
-      <c r="AI165" s="6"/>
-      <c r="AJ165" s="6"/>
-      <c r="AK165" s="6"/>
-      <c r="AL165" s="6"/>
-      <c r="AM165" s="6"/>
-      <c r="AN165" s="9"/>
-      <c r="AO165" s="6"/>
+      <c r="M165" s="5">
+        <v>2150.9400000000001</v>
+      </c>
+      <c r="N165" s="6">
+        <v>27</v>
+      </c>
+      <c r="O165" s="6">
+        <v>14</v>
+      </c>
+      <c r="P165" s="7">
+        <v>3.4294884615384618</v>
+      </c>
+      <c r="Q165" s="8">
+        <v>14.611907142857143</v>
+      </c>
+      <c r="R165" s="8">
+        <v>3.6452357142857141</v>
+      </c>
+      <c r="S165" s="8">
+        <v>7</v>
+      </c>
+      <c r="T165" s="9">
+        <v>0.5714285714285714</v>
+      </c>
+      <c r="U165" s="9">
+        <v>0</v>
+      </c>
+      <c r="V165" s="9">
+        <v>0</v>
+      </c>
+      <c r="W165" s="9">
+        <v>0</v>
+      </c>
+      <c r="X165" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y165" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z165" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA165" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB165" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC165" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AE165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AF165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM165" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN165" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO165" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP165" s="4">
         <v>58</v>
       </c>

</xml_diff>